<commit_message>
PPRA price schedules by default, budgets per line, and the currency follows the country
- Bid packages use the column headings of a PPRA (Kenya) price schedule (Item No, Description,
  Unit, Quantity, Unit Price, Total Price), with a fixed table of the headings other entities use
  ("Rate in KES (VAT inclusive)" is the unit price); anything else is still refused
- Optional budget per BoQ line: the report shows each quote against it
- Each bid file finding states what PPRA's standard tender document for goods says about it
- The currency defaults to the country's; --currency still overrides it
- README: why a price survey is a step in the PPRA procedure (ITT 36), and the Kenyan data limit
</commit_message>
<xml_diff>
--- a/examples/bid-package.xlsx
+++ b/examples/bid-package.xlsx
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,23 +420,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>line</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>item</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>quantity</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Budget per unit</t>
         </is>
       </c>
     </row>
@@ -445,8 +467,16 @@
           <t>Toyota Hilux double cabin pickup</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100000000</v>
       </c>
     </row>
     <row r="3">
@@ -458,8 +488,16 @@
           <t>Laptop computer</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>20</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2400000</v>
       </c>
     </row>
     <row r="4">
@@ -471,8 +509,16 @@
           <t>Motorcycle 125cc</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>10</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1300000</v>
       </c>
     </row>
   </sheetData>
@@ -486,28 +532,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>line</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>unit_price</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>total</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total Price</t>
         </is>
       </c>
     </row>
@@ -515,13 +579,23 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Toyota Hilux double cabin pickup</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
         <v>95000000</v>
       </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>190000000</v>
       </c>
     </row>
@@ -529,13 +603,23 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Laptop computer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" t="n">
         <v>2500000</v>
       </c>
-      <c r="C3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>50000000</v>
       </c>
     </row>
@@ -543,13 +627,23 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Motorcycle 125cc</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="n">
         <v>1300000</v>
       </c>
-      <c r="C4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D4" t="n">
+      <c r="F4" t="n">
         <v>13000000</v>
       </c>
     </row>
@@ -564,28 +658,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>line</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>unit_price</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>total</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total Price</t>
         </is>
       </c>
     </row>
@@ -593,13 +705,23 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Toyota Hilux double cabin pickup</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
         <v>300000000</v>
       </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>600000000</v>
       </c>
     </row>
@@ -607,13 +729,23 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Laptop computer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" t="n">
         <v>2600000</v>
       </c>
-      <c r="C3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>56000000</v>
       </c>
     </row>
@@ -621,13 +753,23 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Motorcycle 125cc</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="n">
         <v>1250000</v>
       </c>
-      <c r="C4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D4" t="n">
+      <c r="F4" t="n">
         <v>12500000</v>
       </c>
     </row>
@@ -642,28 +784,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>line</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>unit_price</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>total</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total Price</t>
         </is>
       </c>
     </row>
@@ -671,13 +831,23 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Toyota Hilux double cabin pickup</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
         <v>95000000</v>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>95000000</v>
       </c>
     </row>
@@ -685,13 +855,23 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Laptop computer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" t="n">
         <v>2500000</v>
       </c>
-      <c r="C3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>50000000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
One workbook per tender: tick off documents, check bids, compare prices
- A Documents sheet (documents in json): the tender's required documents, one rule each
  (Submitted, Valid on YYYY-MM-DD, Covers YYYY-YYYY), and the committee's tick per bidder;
  read strictly, and findings for documents not submitted, expired or missing years
- The report shows each bidder's documents result and a Documents sheet with the checklist
- fairprice --template FILE writes a blank tender workbook (or json, or csv)
- Findings state facts only; no country's legal wording
</commit_message>
<xml_diff>
--- a/examples/bid-package.xlsx
+++ b/examples/bid-package.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="BoQ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bidder A" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Bidder B" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Bidder C" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Documents" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bidder A" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Bidder B" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Bidder C" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -532,46 +533,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item No</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Document</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Rule</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Bidder A</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Unit Price</t>
+          <t>Bidder B</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Total Price</t>
+          <t>Bidder C</t>
         </is>
       </c>
     </row>
@@ -581,22 +582,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Toyota Hilux double cabin pickup</t>
+          <t>Form of Tender, signed and stamped</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="n">
-        <v>95000000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>190000000</v>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -605,22 +612,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Laptop computer</t>
+          <t>Tender security</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>50000000</v>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -629,22 +642,58 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Motorcycle 125cc</t>
+          <t>Tax compliance certificate</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1300000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>13000000</v>
+          <t>Valid on 2025-10-15</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tax clearance certificate</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Covers 2022-2024</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2022-2024</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2022-2024</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2023-2024</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -719,10 +768,10 @@
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>300000000</v>
+        <v>95000000</v>
       </c>
       <c r="F2" t="n">
-        <v>600000000</v>
+        <v>190000000</v>
       </c>
     </row>
     <row r="3">
@@ -743,10 +792,10 @@
         <v>20</v>
       </c>
       <c r="E3" t="n">
-        <v>2600000</v>
+        <v>2500000</v>
       </c>
       <c r="F3" t="n">
-        <v>56000000</v>
+        <v>50000000</v>
       </c>
     </row>
     <row r="4">
@@ -767,10 +816,10 @@
         <v>10</v>
       </c>
       <c r="E4" t="n">
-        <v>1250000</v>
+        <v>1300000</v>
       </c>
       <c r="F4" t="n">
-        <v>12500000</v>
+        <v>13000000</v>
       </c>
     </row>
   </sheetData>
@@ -779,6 +828,132 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Toyota Hilux double cabin pickup</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>600000000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Laptop computer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2600000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>56000000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Motorcycle 125cc</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1250000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>12500000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Back to the bid package: prices only, no documents checklist
The documents checklist is the unpublished half of the brief (no real tender documents
exist to test it on). It is kept on the documents-checklist branch.
</commit_message>
<xml_diff>
--- a/examples/bid-package.xlsx
+++ b/examples/bid-package.xlsx
@@ -8,10 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="BoQ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Documents" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Bidder A" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Bidder B" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Bidder C" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Bidder A" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bidder B" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Bidder C" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -533,46 +532,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ref</t>
+          <t>Item No</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Rule</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Bidder A</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Bidder B</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Bidder C</t>
+          <t>Total Price</t>
         </is>
       </c>
     </row>
@@ -582,28 +581,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Form of Tender, signed and stamped</t>
+          <t>Toyota Hilux double cabin pickup</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Submitted</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>95000000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>190000000</v>
       </c>
     </row>
     <row r="3">
@@ -612,28 +605,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tender security</t>
+          <t>Laptop computer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Submitted</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>50000000</v>
       </c>
     </row>
     <row r="4">
@@ -642,58 +629,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tax compliance certificate</t>
+          <t>Motorcycle 125cc</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Valid on 2025-10-15</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2025-09-30</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-03-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Tax clearance certificate</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Covers 2022-2024</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2022-2024</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2022-2024</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2023-2024</t>
-        </is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1300000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>13000000</v>
       </c>
     </row>
   </sheetData>
@@ -768,10 +719,10 @@
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>95000000</v>
+        <v>300000000</v>
       </c>
       <c r="F2" t="n">
-        <v>190000000</v>
+        <v>600000000</v>
       </c>
     </row>
     <row r="3">
@@ -792,10 +743,10 @@
         <v>20</v>
       </c>
       <c r="E3" t="n">
-        <v>2500000</v>
+        <v>2600000</v>
       </c>
       <c r="F3" t="n">
-        <v>50000000</v>
+        <v>56000000</v>
       </c>
     </row>
     <row r="4">
@@ -816,10 +767,10 @@
         <v>10</v>
       </c>
       <c r="E4" t="n">
-        <v>1300000</v>
+        <v>1250000</v>
       </c>
       <c r="F4" t="n">
-        <v>13000000</v>
+        <v>12500000</v>
       </c>
     </row>
   </sheetData>
@@ -828,132 +779,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item No</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Unit Price</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Total Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Toyota Hilux double cabin pickup</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="n">
-        <v>300000000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>600000000</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Laptop computer</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2600000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>56000000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Motorcycle 125cc</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1250000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>12500000</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
A one-line example bid package, so a demo run takes a few minutes
examples/: the Toyota Hilux line only, three bidders, with two planted problems (an arithmetic
error, a changed quantity). The eval keeps the 3-line package in evals/packages/, so its rounds
stay comparable.
</commit_message>
<xml_diff>
--- a/examples/bid-package.xlsx
+++ b/examples/bid-package.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -479,48 +479,6 @@
         <v>100000000</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Laptop computer</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2400000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Motorcycle 125cc</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1300000</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -532,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -599,54 +557,6 @@
         <v>190000000</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Laptop computer</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>50000000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Motorcycle 125cc</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1300000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>13000000</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -658,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -722,55 +632,7 @@
         <v>300000000</v>
       </c>
       <c r="F2" t="n">
-        <v>600000000</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Laptop computer</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2600000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>56000000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Motorcycle 125cc</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1250000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>12500000</v>
+        <v>650000000</v>
       </c>
     </row>
   </sheetData>
@@ -784,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -851,30 +713,6 @@
         <v>95000000</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Laptop computer</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>50000000</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>